<commit_message>
Pivot table region update
</commit_message>
<xml_diff>
--- a/bikesales dataset.xlsx
+++ b/bikesales dataset.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="16275" windowHeight="8010" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="16275" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8074" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8075" uniqueCount="57">
   <si>
     <t>ID</t>
   </si>
@@ -217,12 +217,15 @@
   <si>
     <t>Bike Sales Dashboard</t>
   </si>
+  <si>
+    <t>PIVOT TABLE FOR ALL REGION VISUALIZATION</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,8 +256,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -264,6 +275,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -280,13 +297,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -296,12 +316,25 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -712,12 +745,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="292928800"/>
-        <c:axId val="333088520"/>
+        <c:axId val="333413464"/>
+        <c:axId val="333420848"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="292928800"/>
+        <c:axId val="333413464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -753,7 +786,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333088520"/>
+        <c:crossAx val="333420848"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -761,7 +794,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333088520"/>
+        <c:axId val="333420848"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -811,7 +844,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="292928800"/>
+        <c:crossAx val="333413464"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1273,12 +1306,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="358712024"/>
-        <c:axId val="358712416"/>
+        <c:axId val="333700704"/>
+        <c:axId val="333701088"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="358712024"/>
+        <c:axId val="333700704"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1314,7 +1347,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="358712416"/>
+        <c:crossAx val="333701088"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1322,7 +1355,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="358712416"/>
+        <c:axId val="333701088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1372,7 +1405,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="358712024"/>
+        <c:crossAx val="333700704"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2601,12 +2634,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="358712808"/>
-        <c:axId val="358713984"/>
+        <c:axId val="333424144"/>
+        <c:axId val="333796008"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="358712808"/>
+        <c:axId val="333424144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2642,7 +2675,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="358713984"/>
+        <c:crossAx val="333796008"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2650,7 +2683,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="358713984"/>
+        <c:axId val="333796008"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2700,7 +2733,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="358712808"/>
+        <c:crossAx val="333424144"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3832,12 +3865,12 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="333090928"/>
-        <c:axId val="333090144"/>
-        <c:axId val="334425976"/>
+        <c:axId val="333921360"/>
+        <c:axId val="349696976"/>
+        <c:axId val="333952912"/>
       </c:line3DChart>
       <c:catAx>
-        <c:axId val="333090928"/>
+        <c:axId val="333921360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3879,7 +3912,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333090144"/>
+        <c:crossAx val="349696976"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3887,7 +3920,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333090144"/>
+        <c:axId val="349696976"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3937,12 +3970,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333090928"/>
+        <c:crossAx val="333921360"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:serAx>
-        <c:axId val="334425976"/>
+        <c:axId val="333952912"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3983,7 +4016,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333090144"/>
+        <c:crossAx val="349696976"/>
         <c:crosses val="autoZero"/>
       </c:serAx>
       <c:spPr>
@@ -5602,12 +5635,12 @@
         <c:gapWidth val="84"/>
         <c:gapDepth val="53"/>
         <c:shape val="box"/>
-        <c:axId val="333091712"/>
-        <c:axId val="333092104"/>
+        <c:axId val="349698152"/>
+        <c:axId val="349695016"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="333091712"/>
+        <c:axId val="349698152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5643,7 +5676,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333092104"/>
+        <c:crossAx val="349695016"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5651,7 +5684,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333092104"/>
+        <c:axId val="349695016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5661,7 +5694,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="333091712"/>
+        <c:crossAx val="349698152"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -27249,368 +27282,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="G3:H7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="10"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="12" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="3" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="7">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="D1:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="G11:H15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="15">
@@ -27761,7 +27432,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="J3:Q7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="15">
@@ -28058,7 +27729,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A1:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
@@ -28220,7 +27891,267 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="G3:H7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="12" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="3" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="D11:E17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
@@ -28313,6 +28244,108 @@
   </dataFields>
   <chartFormats count="1">
     <chartFormat chart="8" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="D1:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="3" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -28481,7 +28514,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O1001" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O1001" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:O1001"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
@@ -28812,50 +28845,50 @@
     <col min="15" max="15" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="8" t="s">
         <v>28</v>
       </c>
     </row>
@@ -77870,7 +77903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -78003,10 +78036,10 @@
       <c r="B5" s="3">
         <v>1000</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="5"/>
+      <c r="E5" s="6"/>
       <c r="G5" s="2" t="s">
         <v>21</v>
       </c>
@@ -78039,10 +78072,10 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="5"/>
+      <c r="B6" s="6"/>
       <c r="G6" s="2" t="s">
         <v>18</v>
       </c>
@@ -78107,20 +78140,20 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="J8" s="4" t="s">
+      <c r="H8" s="6"/>
+      <c r="J8" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="G9" s="1" t="s">
@@ -78243,16 +78276,16 @@
       <c r="E16" s="3">
         <v>192</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="5"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="5"/>
+      <c r="B17" s="6"/>
       <c r="D17" s="2" t="s">
         <v>37</v>
       </c>
@@ -78261,13 +78294,44 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="5"/>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="A20:D21"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="D5:E5"/>
@@ -78287,81 +78351,81 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6"/>
-      <c r="W1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
     </row>
     <row r="3" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Updated the Dashboard visualization
</commit_message>
<xml_diff>
--- a/bikesales dataset.xlsx
+++ b/bikesales dataset.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="16275" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="16275" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -215,10 +215,10 @@
     <t xml:space="preserve">  Bike Purchase by Commute Distance</t>
   </si>
   <si>
-    <t>Bike Sales Dashboard</t>
+    <t>PIVOT TABLE FOR ALL REGION VISUALIZATION</t>
   </si>
   <si>
-    <t>PIVOT TABLE FOR ALL REGION VISUALIZATION</t>
+    <t>Bike Sales Dashboard Visualization</t>
   </si>
 </sst>
 </file>
@@ -307,6 +307,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -315,10 +319,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -745,12 +745,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="333413464"/>
-        <c:axId val="333420848"/>
+        <c:axId val="325194312"/>
+        <c:axId val="347688368"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="333413464"/>
+        <c:axId val="325194312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -786,7 +786,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333420848"/>
+        <c:crossAx val="347688368"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -794,7 +794,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333420848"/>
+        <c:axId val="347688368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -844,7 +844,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333413464"/>
+        <c:crossAx val="325194312"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1306,12 +1306,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="333700704"/>
-        <c:axId val="333701088"/>
+        <c:axId val="326103528"/>
+        <c:axId val="326031048"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="333700704"/>
+        <c:axId val="326103528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1347,7 +1347,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333701088"/>
+        <c:crossAx val="326031048"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1355,7 +1355,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333701088"/>
+        <c:axId val="326031048"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1405,7 +1405,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333700704"/>
+        <c:crossAx val="326103528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2634,12 +2634,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="333424144"/>
-        <c:axId val="333796008"/>
+        <c:axId val="347408952"/>
+        <c:axId val="347409336"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="333424144"/>
+        <c:axId val="347408952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2675,7 +2675,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333796008"/>
+        <c:crossAx val="347409336"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2683,7 +2683,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="333796008"/>
+        <c:axId val="347409336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2733,7 +2733,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333424144"/>
+        <c:crossAx val="347408952"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3865,12 +3865,12 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="333921360"/>
-        <c:axId val="349696976"/>
-        <c:axId val="333952912"/>
+        <c:axId val="347413528"/>
+        <c:axId val="347400056"/>
+        <c:axId val="347821416"/>
       </c:line3DChart>
       <c:catAx>
-        <c:axId val="333921360"/>
+        <c:axId val="347413528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3912,7 +3912,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="349696976"/>
+        <c:crossAx val="347400056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3920,7 +3920,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="349696976"/>
+        <c:axId val="347400056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3970,12 +3970,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333921360"/>
+        <c:crossAx val="347413528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:serAx>
-        <c:axId val="333952912"/>
+        <c:axId val="347821416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4016,7 +4016,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="349696976"/>
+        <c:crossAx val="347400056"/>
         <c:crosses val="autoZero"/>
       </c:serAx>
       <c:spPr>
@@ -5635,12 +5635,12 @@
         <c:gapWidth val="84"/>
         <c:gapDepth val="53"/>
         <c:shape val="box"/>
-        <c:axId val="349698152"/>
-        <c:axId val="349695016"/>
+        <c:axId val="347401624"/>
+        <c:axId val="347402016"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="349698152"/>
+        <c:axId val="347401624"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5676,7 +5676,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="349695016"/>
+        <c:crossAx val="347402016"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5684,7 +5684,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="349695016"/>
+        <c:axId val="347402016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5694,7 +5694,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="349698152"/>
+        <c:crossAx val="347401624"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -27282,6 +27282,377 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="G3:H7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="12" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="3" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
+  <location ref="D11:E17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="8" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="G11:H15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="15">
@@ -27432,7 +27803,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="J3:Q7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="15">
@@ -27729,7 +28100,109 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="D1:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A1:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
@@ -27860,479 +28333,6 @@
     </i>
     <i>
       <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A11:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="G3:H7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="10"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="12" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="3" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="7">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
-  <location ref="D11:E17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Purchased Bike" fld="12" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="8" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="D1:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
     </i>
     <i t="grand">
       <x/>
@@ -28845,50 +28845,50 @@
     <col min="15" max="15" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="5" t="s">
         <v>28</v>
       </c>
     </row>
@@ -78036,10 +78036,10 @@
       <c r="B5" s="3">
         <v>1000</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="6"/>
+      <c r="E5" s="8"/>
       <c r="G5" s="2" t="s">
         <v>21</v>
       </c>
@@ -78072,10 +78072,10 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="8"/>
       <c r="G6" s="2" t="s">
         <v>18</v>
       </c>
@@ -78140,20 +78140,20 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H8" s="6"/>
-      <c r="J8" s="5" t="s">
+      <c r="H8" s="8"/>
+      <c r="J8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="G9" s="1" t="s">
@@ -78276,16 +78276,16 @@
       <c r="E16" s="3">
         <v>192</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="6"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="6"/>
+      <c r="B17" s="8"/>
       <c r="D17" s="2" t="s">
         <v>37</v>
       </c>
@@ -78294,25 +78294,25 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="8"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
+      <c r="A20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
       <c r="E20" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
       <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -78331,14 +78331,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A20:D21"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId8"/>
@@ -78351,81 +78351,81 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
+      <c r="A1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-      <c r="S2" s="7"/>
-      <c r="T2" s="7"/>
-      <c r="U2" s="7"/>
-      <c r="V2" s="7"/>
-      <c r="W2" s="7"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
+      <c r="U2" s="9"/>
+      <c r="V2" s="9"/>
+      <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="7"/>
-      <c r="U3" s="7"/>
-      <c r="V3" s="7"/>
-      <c r="W3" s="7"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
+      <c r="W3" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>